<commit_message>
Corrida | SFE-OLEO | 2026-06-17 12:05:37.633049
</commit_message>
<xml_diff>
--- a/indicadores/SFE-OLEO_out.xlsx
+++ b/indicadores/SFE-OLEO_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="549">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Molienda de soja y girasol en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Molienda de soja y girasol</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">21/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2157,9 +2163,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2170,7 +2180,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2184,12 +2194,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.165882825214336</v>
+        <v>0.161936574491982</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2200,7 +2210,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2228,7 +2238,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2242,12 +2252,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.0115482522177136</v>
+        <v>0.0113010897936541</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2270,7 +2280,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2284,7 +2294,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2298,7 +2308,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2312,12 +2322,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.391973683135439</v>
+        <v>0.448688298447686</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2328,7 +2338,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2342,12 +2352,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.899197748921033</v>
+        <v>0.88757982424164</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2490,10 +2500,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2506,10 +2516,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2533,66 +2543,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>91.0307830435426</v>
@@ -2645,7 +2655,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>84.8620300197529</v>
@@ -2702,7 +2712,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>47.6255853404424</v>
@@ -2759,7 +2769,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>76.2023427508567</v>
@@ -2816,7 +2826,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>133.084486915993</v>
@@ -2873,7 +2883,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>137.672413079316</v>
@@ -2930,7 +2940,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>129.621766846324</v>
@@ -2987,7 +2997,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>131.149957754025</v>
@@ -3044,7 +3054,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>101.453481834509</v>
@@ -3101,7 +3111,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>119.47455726039</v>
@@ -3158,7 +3168,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>119.620431541107</v>
@@ -3215,7 +3225,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>78.0476149758911</v>
@@ -3272,7 +3282,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>94.1893190403374</v>
@@ -3331,7 +3341,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>98.2992440332372</v>
@@ -3390,7 +3400,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>57.0845006188379</v>
@@ -3449,7 +3459,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>74.7116468988395</v>
@@ -3508,7 +3518,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>128.241192156756</v>
@@ -3567,7 +3577,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>133.140919859872</v>
@@ -3626,7 +3636,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>138.021131507809</v>
@@ -3685,7 +3695,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>134.746929192476</v>
@@ -3744,7 +3754,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>142.281593276238</v>
@@ -3803,7 +3813,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>142.695935846138</v>
@@ -3862,7 +3872,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>133.683606567831</v>
@@ -3921,7 +3931,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>73.62228865834</v>
@@ -3980,7 +3990,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>118.902972556647</v>
@@ -4039,7 +4049,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>96.4370350596559</v>
@@ -4098,7 +4108,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>68.6968865065546</v>
@@ -4157,7 +4167,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>89.5035542990138</v>
@@ -4216,7 +4226,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>148.196268398028</v>
@@ -4275,7 +4285,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>146.298146997975</v>
@@ -4334,7 +4344,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>153.810123218605</v>
@@ -4393,7 +4403,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>153.982045953746</v>
@@ -4452,7 +4462,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>150.457231986789</v>
@@ -4511,7 +4521,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>152.390678090598</v>
@@ -4570,7 +4580,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>148.710725214448</v>
@@ -4629,7 +4639,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>129.672739497113</v>
@@ -4688,7 +4698,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>130.313142459618</v>
@@ -4747,7 +4757,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>120.248865028108</v>
@@ -4806,7 +4816,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>86.5584468596617</v>
@@ -4865,7 +4875,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>110.661364730572</v>
@@ -4924,7 +4934,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>149.850627969312</v>
@@ -4983,7 +4993,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>151.072035651305</v>
@@ -5042,7 +5052,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>159.571725924284</v>
@@ -5101,7 +5111,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>162.606641183416</v>
@@ -5160,7 +5170,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>160.432136951875</v>
@@ -5219,7 +5229,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>167.624746440646</v>
@@ -5278,7 +5288,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>162.312483083802</v>
@@ -5337,7 +5347,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>118.242261600878</v>
@@ -5396,7 +5406,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>99.3983806875965</v>
@@ -5455,7 +5465,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>91.1654396114548</v>
@@ -5514,7 +5524,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>84.1885355663584</v>
@@ -5573,7 +5583,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>137.737040533048</v>
@@ -5632,7 +5642,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>174.116278258908</v>
@@ -5691,7 +5701,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>181.226219931192</v>
@@ -5750,7 +5760,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>191.82715120587</v>
@@ -5809,7 +5819,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>213.97987269968</v>
@@ -5868,7 +5878,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>196.801385692165</v>
@@ -5927,7 +5937,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>181.532441611844</v>
@@ -5986,7 +5996,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>94.6423445972136</v>
@@ -6045,7 +6055,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>96.4760352199734</v>
@@ -6104,7 +6114,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>106.525167483662</v>
@@ -6163,7 +6173,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>69.6311876039364</v>
@@ -6222,7 +6232,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>103.410343701858</v>
@@ -6281,7 +6291,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>203.152534318074</v>
@@ -6340,7 +6350,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>231.515735543571</v>
@@ -6399,7 +6409,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>248.161115955958</v>
@@ -6458,7 +6468,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>272.824282236746</v>
@@ -6517,7 +6527,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>261.978529963758</v>
@@ -6576,7 +6586,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>270.249860888513</v>
@@ -6635,7 +6645,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>248.148513910586</v>
@@ -6694,7 +6704,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>244.817038928722</v>
@@ -6753,7 +6763,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>200.721260702978</v>
@@ -6812,7 +6822,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>198.615786389357</v>
@@ -6871,7 +6881,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>152.479837645022</v>
@@ -6930,7 +6940,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>145.534868878315</v>
@@ -6989,7 +6999,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>248.00144700632</v>
@@ -7048,7 +7058,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>284.854502889687</v>
@@ -7107,7 +7117,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>281.574364263678</v>
@@ -7166,7 +7176,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>283.827556199855</v>
@@ -7225,7 +7235,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>285.385241920768</v>
@@ -7284,7 +7294,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>263.409067808618</v>
@@ -7343,7 +7353,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>256.817794303579</v>
@@ -7402,7 +7412,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>227.18359460004</v>
@@ -7461,7 +7471,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>175.53707174899</v>
@@ -7520,7 +7530,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>207.847020834233</v>
@@ -7579,7 +7589,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>159.328230182421</v>
@@ -7638,7 +7648,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>154.495219713209</v>
@@ -7697,7 +7707,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>264.663504719146</v>
@@ -7756,7 +7766,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>280.677157627288</v>
@@ -7815,7 +7825,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>248.895556692704</v>
@@ -7874,7 +7884,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>262.647215296086</v>
@@ -7933,7 +7943,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>274.697134592186</v>
@@ -7992,7 +8002,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>255.99874915623</v>
@@ -8051,7 +8061,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>235.764544954216</v>
@@ -8110,7 +8120,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>231.820900137368</v>
@@ -8169,7 +8179,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>186.556408077395</v>
@@ -8228,7 +8238,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>163.133670959391</v>
@@ -8287,7 +8297,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>77.0551342244605</v>
@@ -8346,7 +8356,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>160.359237792984</v>
@@ -8405,7 +8415,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>258.665631495046</v>
@@ -8464,7 +8474,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>267.499114182882</v>
@@ -8523,7 +8533,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>249.315309076678</v>
@@ -8582,7 +8592,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>275.018899485795</v>
@@ -8641,7 +8651,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>277.391550263312</v>
@@ -8700,7 +8710,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>244.261523914057</v>
@@ -8759,7 +8769,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>263.303785732653</v>
@@ -8818,7 +8828,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>259.385853509854</v>
@@ -8877,7 +8887,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>235.201771734261</v>
@@ -8936,7 +8946,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>210.746144196846</v>
@@ -8995,7 +9005,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>139.940357029458</v>
@@ -9054,7 +9064,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>188.669338022084</v>
@@ -9113,7 +9123,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>250.213381938301</v>
@@ -9172,7 +9182,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>305.05699704429</v>
@@ -9231,7 +9241,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>305.88016131325</v>
@@ -9290,7 +9300,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>321.203029348723</v>
@@ -9349,7 +9359,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>317.998161736875</v>
@@ -9408,7 +9418,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>317.01372866562</v>
@@ -9467,7 +9477,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>315.076502413618</v>
@@ -9526,7 +9536,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>272.955685022824</v>
@@ -9585,7 +9595,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>265.977817646611</v>
@@ -9644,7 +9654,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>255.472620768087</v>
@@ -9703,7 +9713,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>219.798508822703</v>
@@ -9762,7 +9772,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>263.977540121518</v>
@@ -9821,7 +9831,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>310.22636778683</v>
@@ -9880,7 +9890,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>332.178566187137</v>
@@ -9939,7 +9949,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>325.321104762478</v>
@@ -9998,7 +10008,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>347.725752338248</v>
@@ -10057,7 +10067,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>322.039727737869</v>
@@ -10116,7 +10126,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>328.135870536246</v>
@@ -10175,7 +10185,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>347.617161544808</v>
@@ -10234,7 +10244,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>318.02322805166</v>
@@ -10293,7 +10303,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>289.727543643924</v>
@@ -10352,7 +10362,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>312.780416288914</v>
@@ -10411,7 +10421,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>234.994311844402</v>
@@ -10470,7 +10480,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>249.23108365534</v>
@@ -10529,7 +10539,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>328.188217327205</v>
@@ -10588,7 +10598,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>362.639666703273</v>
@@ -10647,7 +10657,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>346.497221463686</v>
@@ -10706,7 +10716,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>329.539403569541</v>
@@ -10765,7 +10775,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>326.420716174278</v>
@@ -10824,7 +10834,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>305.388450225693</v>
@@ -10883,7 +10893,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>308.085525747412</v>
@@ -10942,7 +10952,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>287.640258382967</v>
@@ -11001,7 +11011,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>239.937475676394</v>
@@ -11060,7 +11070,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>327.674059357113</v>
@@ -11119,7 +11129,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>303.846110575858</v>
@@ -11178,7 +11188,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>323.495119690969</v>
@@ -11237,7 +11247,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>340.999383589591</v>
@@ -11296,7 +11306,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>413.155165008039</v>
@@ -11355,7 +11365,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>414.381199796828</v>
@@ -11414,7 +11424,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>441.042481171687</v>
@@ -11473,7 +11483,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>405.359232693644</v>
@@ -11532,7 +11542,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>418.617542549492</v>
@@ -11591,7 +11601,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>346.53856163168</v>
@@ -11650,7 +11660,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>293.901786549829</v>
@@ -11709,7 +11719,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>387.655030901033</v>
@@ -11768,7 +11778,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>413.279365720198</v>
@@ -11827,7 +11837,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>333.292154403574</v>
@@ -11886,7 +11896,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>383.15879935169</v>
@@ -11945,7 +11955,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>478.583545891942</v>
@@ -12004,7 +12014,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>524.522880511251</v>
@@ -12063,7 +12073,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>486.378486531449</v>
@@ -12122,7 +12132,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>483.254543292638</v>
@@ -12181,7 +12191,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>439.942180877148</v>
@@ -12240,7 +12250,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>462.988382411712</v>
@@ -12299,7 +12309,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>417.686800527384</v>
@@ -12358,7 +12368,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>404.633137982852</v>
@@ -12417,7 +12427,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>414.811256464842</v>
@@ -12476,7 +12486,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>404.700752663151</v>
@@ -12535,7 +12545,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>337.687623651799</v>
@@ -12594,7 +12604,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>411.728602386644</v>
@@ -12653,7 +12663,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>490.372343958352</v>
@@ -12712,7 +12722,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>542.829122871666</v>
@@ -12771,7 +12781,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>510.007184050454</v>
@@ -12830,7 +12840,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>452.147207376816</v>
@@ -12889,7 +12899,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>469.009544486136</v>
@@ -12948,7 +12958,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>548.786213483115</v>
@@ -13007,7 +13017,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>562.642778136947</v>
@@ -13066,7 +13076,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>525.794804176502</v>
@@ -13125,7 +13135,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>555.126420677023</v>
@@ -13184,7 +13194,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>482.736770502289</v>
@@ -13243,7 +13253,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>365.763254558947</v>
@@ -13302,7 +13312,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>232.511727792053</v>
@@ -13361,7 +13371,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>492.913569656802</v>
@@ -13420,7 +13430,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>563.278659416076</v>
@@ -13479,7 +13489,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>328.331255193453</v>
@@ -13538,7 +13548,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>574.044616542959</v>
@@ -13597,7 +13607,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>496.776503852704</v>
@@ -13656,7 +13666,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>523.032609309416</v>
@@ -13715,7 +13725,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>444.476876535906</v>
@@ -13774,7 +13784,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>387.827154321377</v>
@@ -13833,7 +13843,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>374.970706669512</v>
@@ -13892,7 +13902,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>399.697488620965</v>
@@ -13951,7 +13961,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>346.056880612487</v>
@@ -14010,7 +14020,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>360.029623318291</v>
@@ -14069,7 +14079,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>536.495494514456</v>
@@ -14128,7 +14138,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>589.302631565878</v>
@@ -14187,7 +14197,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>504.829121473604</v>
@@ -14246,7 +14256,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>451.892561873458</v>
@@ -14305,7 +14315,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>350.355435950338</v>
@@ -14364,7 +14374,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>370.925798325194</v>
@@ -14423,7 +14433,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>381.648618668618</v>
@@ -14482,7 +14492,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>357.083425284802</v>
@@ -14541,7 +14551,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>310.100977190955</v>
@@ -14600,7 +14610,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>266.245694153085</v>
@@ -14659,7 +14669,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>214.106753487717</v>
@@ -14718,7 +14728,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>287.615283739774</v>
@@ -14777,7 +14787,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>579.945311704624</v>
@@ -14836,7 +14846,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>620.160391700821</v>
@@ -14895,7 +14905,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>534.559223920624</v>
@@ -14954,7 +14964,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>511.73686256975</v>
@@ -15013,7 +15023,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>589.092155783701</v>
@@ -15072,7 +15082,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>554.726776085561</v>
@@ -15131,7 +15141,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>548.664917483569</v>
@@ -15190,7 +15200,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>468.544961802511</v>
@@ -15249,7 +15259,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>403.808742883489</v>
@@ -15308,7 +15318,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>365.135865908603</v>
@@ -15367,7 +15377,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>313.74253378602</v>
@@ -15426,7 +15436,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>472.56270610022</v>
@@ -15485,7 +15495,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>590.152415161741</v>
@@ -15544,7 +15554,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>617.777007699319</v>
@@ -15603,7 +15613,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>519.548264732001</v>
@@ -15662,7 +15672,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>496.570305145063</v>
@@ -15721,7 +15731,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>467.02249512481</v>
@@ -15780,7 +15790,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>579.357438901155</v>
@@ -15839,7 +15849,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>510.673953319824</v>
@@ -15898,7 +15908,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>455.128706314736</v>
@@ -15957,7 +15967,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>425.406593222593</v>
@@ -16016,7 +16026,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>416.768351816331</v>
@@ -16075,7 +16085,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>368.266472392545</v>
@@ -16134,7 +16144,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>391.083020584574</v>
@@ -16193,7 +16203,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>576.211470000802</v>
@@ -16252,7 +16262,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>587.26927287989</v>
@@ -16311,7 +16321,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>494.694339393308</v>
@@ -16370,7 +16380,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>444.629060257843</v>
@@ -16429,7 +16439,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>410.521538620132</v>
@@ -16488,7 +16498,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>453.804265870542</v>
@@ -16547,7 +16557,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>347.341338146423</v>
@@ -16606,7 +16616,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>323.205797904357</v>
@@ -16665,7 +16675,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>279.357804392475</v>
@@ -16724,7 +16734,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>284.146155292045</v>
@@ -16783,7 +16793,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>198.172394064637</v>
@@ -16842,7 +16852,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>277.507808748013</v>
@@ -16901,7 +16911,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>542.570739265968</v>
@@ -16960,7 +16970,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>591.793721580268</v>
@@ -17019,7 +17029,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>601.266081378227</v>
@@ -17078,7 +17088,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>557.107114156125</v>
@@ -17137,7 +17147,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>545.789211532518</v>
@@ -17196,7 +17206,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>551.470869850403</v>
@@ -17255,7 +17265,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>443.360698571621</v>
@@ -17314,7 +17324,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>354.803647622686</v>
@@ -17373,7 +17383,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>250.660396557804</v>
@@ -17432,7 +17442,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>295.998755240939</v>
@@ -17491,7 +17501,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>239.367735682956</v>
@@ -17550,7 +17560,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>328.639690820364</v>
@@ -17609,7 +17619,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>608.094591804874</v>
@@ -17668,7 +17678,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>712.536250559267</v>
@@ -17727,7 +17737,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>646.067167158672</v>
@@ -17786,7 +17796,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>578.134770787774</v>
@@ -17845,7 +17855,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>523.876291471574</v>
@@ -17904,7 +17914,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>497.665689948175</v>
@@ -17963,7 +17973,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>451.463122476474</v>
@@ -18022,7 +18032,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>454.959739320081</v>
@@ -18081,7 +18091,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>359.972364140163</v>
@@ -18140,7 +18150,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>275.916739874625</v>
@@ -18199,7 +18209,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>313.890817751279</v>
@@ -18258,7 +18268,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>367.360561137447</v>
@@ -18317,7 +18327,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>664.332722706789</v>
@@ -18376,7 +18386,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>547.658745518148</v>
@@ -18435,7 +18445,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>694.735394279507</v>
@@ -18494,7 +18504,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>736.775971860965</v>
@@ -18553,7 +18563,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>647.714925919855</v>
@@ -18612,7 +18622,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>577.807068930734</v>
@@ -18671,7 +18681,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>578.237276182538</v>
@@ -18730,7 +18740,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>462.682858355784</v>
@@ -18789,7 +18799,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>413.458730169214</v>
@@ -18848,7 +18858,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>611.624759649174</v>
@@ -18907,7 +18917,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>506.98661277265</v>
@@ -18966,7 +18976,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>524.057372576041</v>
@@ -19025,7 +19035,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>596.127321611864</v>
@@ -19084,7 +19094,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>668.322426736399</v>
@@ -19143,7 +19153,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>639.16195350998</v>
@@ -19202,7 +19212,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>610.764132791219</v>
@@ -19261,7 +19271,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>567.809585808396</v>
@@ -19320,7 +19330,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>519.304840418924</v>
@@ -19379,7 +19389,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>545.475306942253</v>
@@ -19438,7 +19448,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>569.134310909474</v>
@@ -19497,7 +19507,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>504.034065804576</v>
@@ -19556,7 +19566,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>467.897590522429</v>
@@ -19615,7 +19625,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>422.835971880452</v>
@@ -19674,7 +19684,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>541.339871019626</v>
@@ -19733,7 +19743,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>646.188892860679</v>
@@ -19792,7 +19802,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>707.679368376107</v>
@@ -19851,7 +19861,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>582.376650297014</v>
@@ -19910,7 +19920,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>665.344438489119</v>
@@ -19969,7 +19979,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>566.580257123841</v>
@@ -20028,7 +20038,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>513.863269986605</v>
@@ -20087,7 +20097,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>540.226216946293</v>
@@ -20146,7 +20156,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>466.904958587163</v>
@@ -20205,7 +20215,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>305.98562219969</v>
@@ -20264,7 +20274,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>449.437174268531</v>
@@ -20323,7 +20333,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>379.574934419493</v>
@@ -20382,7 +20392,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>495.190993224233</v>
@@ -20441,7 +20451,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>539.021924267151</v>
@@ -20500,7 +20510,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>584.430380037717</v>
@@ -20559,7 +20569,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>510.420474686774</v>
@@ -20618,7 +20628,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>532.977630661613</v>
@@ -20677,7 +20687,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>471.991570204587</v>
@@ -20736,7 +20746,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>454.377316920254</v>
@@ -20795,7 +20805,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>513.397522673415</v>
@@ -20854,7 +20864,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>507.66729815037</v>
@@ -20913,7 +20923,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>420.836182030413</v>
@@ -20972,7 +20982,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>406.777091799849</v>
@@ -21031,7 +21041,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>362.506820208461</v>
@@ -21090,7 +21100,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>475.366912557472</v>
@@ -21149,7 +21159,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>609.447682296114</v>
@@ -21208,7 +21218,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>634.677141264602</v>
@@ -21267,7 +21277,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>681.385285723946</v>
@@ -21326,7 +21336,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>708.347780675341</v>
@@ -21385,7 +21395,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>679.87165204618</v>
@@ -21444,7 +21454,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>485.607925053365</v>
@@ -21503,7 +21513,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>620.449963859869</v>
@@ -21562,7 +21572,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>465.922105681902</v>
@@ -21621,7 +21631,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>416.547640777135</v>
@@ -21680,7 +21690,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>365.88048852692</v>
@@ -21739,7 +21749,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>427.646688698551</v>
@@ -21798,7 +21808,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>440.621196742905</v>
@@ -21857,7 +21867,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>582.565885154922</v>
@@ -21916,7 +21926,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>632.447003734513</v>
@@ -21975,7 +21985,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>559.593784143312</v>
@@ -22034,7 +22044,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>527.638815557407</v>
@@ -22093,7 +22103,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>516.586739967223</v>
@@ -22152,7 +22162,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>508.200498439772</v>
@@ -22211,7 +22221,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>474.904313476834</v>
@@ -22270,7 +22280,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>453.420423957705</v>
@@ -22329,7 +22339,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>95.7628447568809</v>
@@ -22388,7 +22398,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>519.644192343236</v>
@@ -22447,7 +22457,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>457.614200393974</v>
@@ -22506,7 +22516,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>552.008432064173</v>
@@ -22565,7 +22575,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>686.85502305368</v>
@@ -22624,7 +22634,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>690.393174994202</v>
@@ -22683,7 +22693,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>669.645458856943</v>
@@ -22742,7 +22752,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>611.8331137919</v>
@@ -22801,7 +22811,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>565.329716829141</v>
@@ -22860,7 +22870,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>570.830999779926</v>
@@ -22919,7 +22929,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>535.98989762708</v>
@@ -22978,7 +22988,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>441.489623859202</v>
@@ -23037,7 +23047,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>445.554784605466</v>
@@ -23096,7 +23106,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>398.542710302203</v>
@@ -23155,7 +23165,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>429.061084202022</v>
@@ -23214,7 +23224,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>493.071592696233</v>
@@ -23273,7 +23283,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>645.349693497394</v>
@@ -23332,7 +23342,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>676.448413156935</v>
@@ -23391,7 +23401,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>642.082703606435</v>
@@ -23450,7 +23460,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>556.07636452863</v>
@@ -23509,7 +23519,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>483.574665067104</v>
@@ -23568,7 +23578,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>471.342748859452</v>
@@ -23627,7 +23637,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>440.031550234921</v>
@@ -23686,7 +23696,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>507.583630378038</v>
@@ -23745,7 +23755,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>403.371672646819</v>
@@ -23804,7 +23814,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>294.895740094309</v>
@@ -23863,7 +23873,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>251.564731535647</v>
@@ -23922,7 +23932,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>376.622607871584</v>
@@ -23981,7 +23991,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>487.65412951393</v>
@@ -24040,7 +24050,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>564.544251247259</v>
@@ -24099,7 +24109,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>493.017560239736</v>
@@ -24158,7 +24168,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>437.584920110443</v>
@@ -24217,7 +24227,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>323.569875447391</v>
@@ -24276,7 +24286,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>318.511590259523</v>
@@ -24335,7 +24345,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>302.642168647609</v>
@@ -24394,7 +24404,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>298.786759352783</v>
@@ -24453,7 +24463,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>288.591398732223</v>
@@ -24512,7 +24522,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>349.846473961735</v>
@@ -24571,7 +24581,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>404.280806652846</v>
@@ -24630,7 +24640,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>485.029061973218</v>
@@ -24689,7 +24699,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>638.969182651679</v>
@@ -24748,7 +24758,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>639.845918279334</v>
@@ -24807,7 +24817,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>646.538588666314</v>
@@ -24866,7 +24876,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>701.539671423975</v>
@@ -24925,7 +24935,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>509.092743300337</v>
@@ -24984,7 +24994,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>655.502233382336</v>
@@ -25043,7 +25053,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>650.888871277506</v>
@@ -25102,7 +25112,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>562.153959331793</v>
@@ -25161,7 +25171,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>584.550676625874</v>
@@ -25220,7 +25230,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>463.048686352834</v>
@@ -25279,7 +25289,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>433.681073884442</v>
@@ -25338,7 +25348,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>531.731348183607</v>
@@ -25397,7 +25407,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>555.79666634231</v>
@@ -25456,7 +25466,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>632.812702491225</v>
@@ -25515,7 +25525,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B391" s="2" t="n">
         <v>667.181774592755</v>
@@ -25574,7 +25584,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B392" s="2" t="n">
         <v>620.498012726056</v>
@@ -25633,7 +25643,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B393" s="2" t="n">
         <v>636.709375070504</v>
@@ -25692,7 +25702,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B394" s="2" t="n">
         <v>682.520646112063</v>
@@ -25751,7 +25761,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B395" s="2" t="n">
         <v>656.041412385367</v>
@@ -25810,7 +25820,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B396" s="2" t="n">
         <v>577.373484743797</v>
@@ -25869,7 +25879,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B397" s="2" t="n">
         <v>488.89668369853</v>
@@ -25928,7 +25938,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B398" s="2" t="n">
         <v>443.774717241543</v>
@@ -25987,7 +25997,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B399" s="2" t="n">
         <v>319.721570514651</v>
@@ -26046,7 +26056,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B400" s="2" t="n">
         <v>554.907043741628</v>
@@ -26105,7 +26115,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B401" s="2" t="n">
         <v>596.331356495142</v>
@@ -26164,7 +26174,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3" t="n">
@@ -26197,7 +26207,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3" t="n">
@@ -26230,7 +26240,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3" t="n">
@@ -26263,7 +26273,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3" t="n">
@@ -26296,7 +26306,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3" t="n">
@@ -26329,7 +26339,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3" t="n">
@@ -26362,7 +26372,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3" t="n">
@@ -26395,7 +26405,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3" t="n">
@@ -26428,7 +26438,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3" t="n">
@@ -26461,7 +26471,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3" t="n">
@@ -26494,7 +26504,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3" t="n">
@@ -26527,7 +26537,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3" t="n">
@@ -26560,7 +26570,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -26583,7 +26593,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -26606,7 +26616,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -26629,7 +26639,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -26652,7 +26662,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -26675,7 +26685,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -26698,7 +26708,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -26721,7 +26731,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -26744,7 +26754,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -26767,7 +26777,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -26790,7 +26800,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -26813,7 +26823,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -26836,7 +26846,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -26859,7 +26869,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -26882,7 +26892,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26905,7 +26915,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26928,7 +26938,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26951,7 +26961,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26974,7 +26984,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -26997,7 +27007,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -27020,7 +27030,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -27043,7 +27053,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -27066,7 +27076,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -27089,7 +27099,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -27112,7 +27122,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -27135,7 +27145,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -27158,7 +27168,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -27181,7 +27191,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -27204,7 +27214,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -27227,7 +27237,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -27250,7 +27260,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -27273,7 +27283,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -27296,7 +27306,7 @@
     </row>
     <row r="446">
       <c r="A446" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B446" s="2"/>
       <c r="C446" s="3"/>
@@ -27319,7 +27329,7 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B447" s="2"/>
       <c r="C447" s="3"/>
@@ -27342,7 +27352,7 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B448" s="2"/>
       <c r="C448" s="3"/>
@@ -27365,7 +27375,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B449" s="2"/>
       <c r="C449" s="3"/>
@@ -27388,7 +27398,7 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B450" s="2"/>
       <c r="C450" s="3"/>
@@ -27411,7 +27421,7 @@
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B451" s="2"/>
       <c r="C451" s="3"/>
@@ -27434,7 +27444,7 @@
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B452" s="2"/>
       <c r="C452" s="3"/>
@@ -27457,7 +27467,7 @@
     </row>
     <row r="453">
       <c r="A453" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B453" s="2"/>
       <c r="C453" s="3"/>
@@ -27480,7 +27490,7 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B454" s="2"/>
       <c r="C454" s="3"/>
@@ -27503,7 +27513,7 @@
     </row>
     <row r="455">
       <c r="A455" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B455" s="2"/>
       <c r="C455" s="3"/>
@@ -27526,7 +27536,7 @@
     </row>
     <row r="456">
       <c r="A456" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B456" s="2"/>
       <c r="C456" s="3"/>
@@ -27549,7 +27559,7 @@
     </row>
     <row r="457">
       <c r="A457" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B457" s="2"/>
       <c r="C457" s="3"/>
@@ -27583,97 +27593,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
   </sheetData>
@@ -27697,7 +27707,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -27707,160 +27717,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.010377835661912</v>
+        <v>-0.00947237875186118</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0182050333852851</v>
+        <v>-0.0155293709306641</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.00472084029738783</v>
+        <v>-0.0019088885299252</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0403754961678676</v>
+        <v>0.0425479868940257</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.0979853771239026</v>
+        <v>0.0989877628392053</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.134123152428951</v>
+        <v>0.132245026677275</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.161220322596053</v>
+        <v>0.156972503130772</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.165882825214336</v>
+        <v>0.161936574491982</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.143981542306477</v>
+        <v>0.141143398855577</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.107462794574279</v>
+        <v>0.106306583961926</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.0375851627243077</v>
+        <v>0.0397379602725204</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>-0.0298298404952448</v>
+        <v>-0.0256540219899386</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>-0.042518486095043</v>
+        <v>-0.0382737086169833</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>-0.0392967779676948</v>
+        <v>-0.0370334616867321</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>-0.0365581664944109</v>
+        <v>-0.036253191734937</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.0382988773985596</v>
+        <v>-0.0399130227957304</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0584961870409468</v>
+        <v>-0.0615584333004302</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0661248970613202</v>
+        <v>-0.0696058813806383</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.0651621145973344</v>
+        <v>-0.0666638633309223</v>
       </c>
     </row>
     <row r="24">

</xml_diff>